<commit_message>
feat(table): add category column and drop masked contact links
Add the new "category" field to the sortable/searchable columns and
rebalance fixed column widths to keep the sum at 100%. Recompute the
horizontal-overflow breakpoint to 928px (880px table min-width + 24px
padding per side) and update the matching media queries and
H_SCROLL_QUERY in DirectoryTable.tsx.

Stop rendering phone and email as tel:/mailto: links, since the data
layer masks those values (e.g. 138*****000), producing broken links
that cannot be dialed or emailed. Keep them as plain text and drop the
now-unused .link styles. Also refresh the source xlsx and the CSS
comments documenting the column rationale.
</commit_message>
<xml_diff>
--- a/src/excel/源头厂商.xlsx
+++ b/src/excel/源头厂商.xlsx
@@ -27,11 +27,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="169">
   <si>
     <t>源头厂商</t>
   </si>
   <si>
+    <t>品类</t>
+  </si>
+  <si>
     <t>商品</t>
   </si>
   <si>
@@ -47,16 +50,490 @@
     <t>是否验证</t>
   </si>
   <si>
-    <t>娃哈哈</t>
+    <t>华东饮品供应链</t>
+  </si>
+  <si>
+    <t>饮品</t>
   </si>
   <si>
     <t>矿泉水</t>
   </si>
   <si>
-    <t>wahah@qq.com</t>
-  </si>
-  <si>
-    <t>农夫山泉</t>
+    <t>huadong@example.com</t>
+  </si>
+  <si>
+    <t>是</t>
+  </si>
+  <si>
+    <t>苏打水</t>
+  </si>
+  <si>
+    <t>果汁饮料</t>
+  </si>
+  <si>
+    <t>纯净水</t>
+  </si>
+  <si>
+    <t>川渝调味品集采</t>
+  </si>
+  <si>
+    <t>调味品</t>
+  </si>
+  <si>
+    <t>酿造酱油</t>
+  </si>
+  <si>
+    <t>chuanyu@example.com</t>
+  </si>
+  <si>
+    <t>香醋</t>
+  </si>
+  <si>
+    <t>火锅底料</t>
+  </si>
+  <si>
+    <t>郫县豆瓣</t>
+  </si>
+  <si>
+    <t>岭南果蔬直供</t>
+  </si>
+  <si>
+    <t>生鲜果蔬</t>
+  </si>
+  <si>
+    <t>冷冻玉米粒</t>
+  </si>
+  <si>
+    <t>lingnan@example.com</t>
+  </si>
+  <si>
+    <t>鲜切菠萝</t>
+  </si>
+  <si>
+    <t>白蘑菇</t>
+  </si>
+  <si>
+    <t>老豆腐</t>
+  </si>
+  <si>
+    <t>齐鲁粮油贸易</t>
+  </si>
+  <si>
+    <t>粮油</t>
+  </si>
+  <si>
+    <t>一级大米</t>
+  </si>
+  <si>
+    <t>qilu@example.com</t>
+  </si>
+  <si>
+    <t>高筋面粉</t>
+  </si>
+  <si>
+    <t>花生油</t>
+  </si>
+  <si>
+    <t>龙须挂面</t>
+  </si>
+  <si>
+    <t>云贵茶叶合作社</t>
+  </si>
+  <si>
+    <t>茶叶</t>
+  </si>
+  <si>
+    <t>云雾绿茶</t>
+  </si>
+  <si>
+    <t>yungui@example.com</t>
+  </si>
+  <si>
+    <t>滇红红茶</t>
+  </si>
+  <si>
+    <t>普洱熟茶</t>
+  </si>
+  <si>
+    <t>茉莉花茶</t>
+  </si>
+  <si>
+    <t>闽南水产供应</t>
+  </si>
+  <si>
+    <t>水产</t>
+  </si>
+  <si>
+    <t>冷冻虾仁</t>
+  </si>
+  <si>
+    <t>minnan@example.com</t>
+  </si>
+  <si>
+    <t>带鱼段</t>
+  </si>
+  <si>
+    <t>盐渍海带</t>
+  </si>
+  <si>
+    <t>鱿鱼圈</t>
+  </si>
+  <si>
+    <t>湘鄂食品原料</t>
+  </si>
+  <si>
+    <t>香辛料</t>
+  </si>
+  <si>
+    <t>辣椒粉</t>
+  </si>
+  <si>
+    <t>xiange@example.com</t>
+  </si>
+  <si>
+    <t>否</t>
+  </si>
+  <si>
+    <t>八角</t>
+  </si>
+  <si>
+    <t>桂皮</t>
+  </si>
+  <si>
+    <t>花椒</t>
+  </si>
+  <si>
+    <t>华北乳品供应链</t>
+  </si>
+  <si>
+    <t>乳品</t>
+  </si>
+  <si>
+    <t>纯牛奶</t>
+  </si>
+  <si>
+    <t>huabei@example.com</t>
+  </si>
+  <si>
+    <t>常温酸奶</t>
+  </si>
+  <si>
+    <t>全脂奶粉</t>
+  </si>
+  <si>
+    <t>动物黄油</t>
+  </si>
+  <si>
+    <t>东北杂粮集采</t>
+  </si>
+  <si>
+    <t>杂粮</t>
+  </si>
+  <si>
+    <t>玉米碴</t>
+  </si>
+  <si>
+    <t>dongbei@example.com</t>
+  </si>
+  <si>
+    <t>小米</t>
+  </si>
+  <si>
+    <t>红小豆</t>
+  </si>
+  <si>
+    <t>绿豆</t>
+  </si>
+  <si>
+    <t>江浙休闲食品</t>
+  </si>
+  <si>
+    <t>休闲食品</t>
+  </si>
+  <si>
+    <t>混合坚果</t>
+  </si>
+  <si>
+    <t>jiangzhe@example.com</t>
+  </si>
+  <si>
+    <t>话梅蜜饯</t>
+  </si>
+  <si>
+    <t>苏打饼干</t>
+  </si>
+  <si>
+    <t>猪肉脯</t>
+  </si>
+  <si>
+    <t>西北干果贸易</t>
+  </si>
+  <si>
+    <t>干果</t>
+  </si>
+  <si>
+    <t>和田红枣</t>
+  </si>
+  <si>
+    <t>xibei@example.com</t>
+  </si>
+  <si>
+    <t>葡萄干</t>
+  </si>
+  <si>
+    <t>核桃仁</t>
+  </si>
+  <si>
+    <t>宁夏枸杞</t>
+  </si>
+  <si>
+    <t>珠三角日化供应</t>
+  </si>
+  <si>
+    <t>日化</t>
+  </si>
+  <si>
+    <t>洗洁精</t>
+  </si>
+  <si>
+    <t>zhusanjiao@example.com</t>
+  </si>
+  <si>
+    <t>洗衣液</t>
+  </si>
+  <si>
+    <t>抽纸</t>
+  </si>
+  <si>
+    <t>垃圾袋</t>
+  </si>
+  <si>
+    <t>中原面点原料</t>
+  </si>
+  <si>
+    <t>面点原料</t>
+  </si>
+  <si>
+    <t>速冻面团</t>
+  </si>
+  <si>
+    <t>zhongyuan@example.com</t>
+  </si>
+  <si>
+    <t>高活性酵母</t>
+  </si>
+  <si>
+    <t>泡打粉</t>
+  </si>
+  <si>
+    <t>糖粉</t>
+  </si>
+  <si>
+    <t>海南热带果品</t>
+  </si>
+  <si>
+    <t>热带水果</t>
+  </si>
+  <si>
+    <t>椰青</t>
+  </si>
+  <si>
+    <t>hainan@example.com</t>
+  </si>
+  <si>
+    <t>芒果</t>
+  </si>
+  <si>
+    <t>菠萝</t>
+  </si>
+  <si>
+    <t>香蕉</t>
+  </si>
+  <si>
+    <t>皖南干货贸易</t>
+  </si>
+  <si>
+    <t>干货</t>
+  </si>
+  <si>
+    <t>黑木耳</t>
+  </si>
+  <si>
+    <t>wannan@example.com</t>
+  </si>
+  <si>
+    <t>香菇干</t>
+  </si>
+  <si>
+    <t>笋干</t>
+  </si>
+  <si>
+    <t>腐竹</t>
+  </si>
+  <si>
+    <t>安克</t>
+  </si>
+  <si>
+    <t>消费电子</t>
+  </si>
+  <si>
+    <t>快充充电器</t>
+  </si>
+  <si>
+    <t>anker@example.com</t>
+  </si>
+  <si>
+    <t>大疆</t>
+  </si>
+  <si>
+    <t>消费级无人机</t>
+  </si>
+  <si>
+    <t>dji@example.com</t>
+  </si>
+  <si>
+    <t>扫地机器人</t>
+  </si>
+  <si>
+    <t>xiaomi@example.com</t>
+  </si>
+  <si>
+    <t>正浩</t>
+  </si>
+  <si>
+    <t>户外储能</t>
+  </si>
+  <si>
+    <t>户外储能电源</t>
+  </si>
+  <si>
+    <t>ecoflow@example.com</t>
+  </si>
+  <si>
+    <t>九号</t>
+  </si>
+  <si>
+    <t>电动滑板车</t>
+  </si>
+  <si>
+    <t>segway@example.com</t>
+  </si>
+  <si>
+    <t>深圳清洁机器人供应链</t>
+  </si>
+  <si>
+    <t>泳池机器人</t>
+  </si>
+  <si>
+    <t>shenzhen-clean@example.com</t>
+  </si>
+  <si>
+    <t>许昌发制品供应链</t>
+  </si>
+  <si>
+    <t>服饰配饰</t>
+  </si>
+  <si>
+    <t>假发</t>
+  </si>
+  <si>
+    <t>xuchang@example.com</t>
+  </si>
+  <si>
+    <t>义乌美妆配饰供应链</t>
+  </si>
+  <si>
+    <t>假睫毛</t>
+  </si>
+  <si>
+    <t>yiwu@example.com</t>
+  </si>
+  <si>
+    <t>穿戴甲</t>
+  </si>
+  <si>
+    <t>泡泡玛特</t>
+  </si>
+  <si>
+    <t>玩具潮玩</t>
+  </si>
+  <si>
+    <t>潮玩盲盒</t>
+  </si>
+  <si>
+    <t>popmart@example.com</t>
+  </si>
+  <si>
+    <t>好孩子</t>
+  </si>
+  <si>
+    <t>婴儿推车</t>
+  </si>
+  <si>
+    <t>goodbaby@example.com</t>
+  </si>
+  <si>
+    <t>宁波家居用品供应链</t>
+  </si>
+  <si>
+    <t>家居日用</t>
+  </si>
+  <si>
+    <t>仿真绿植</t>
+  </si>
+  <si>
+    <t>ningbo@example.com</t>
+  </si>
+  <si>
+    <t>圣诞装饰</t>
+  </si>
+  <si>
+    <t>户外桌椅</t>
+  </si>
+  <si>
+    <t>美的</t>
+  </si>
+  <si>
+    <t>厨房小家电</t>
+  </si>
+  <si>
+    <t>空气炸锅</t>
+  </si>
+  <si>
+    <t>midea@example.com</t>
+  </si>
+  <si>
+    <t>柳州特色食品供应链</t>
+  </si>
+  <si>
+    <t>特色食品</t>
+  </si>
+  <si>
+    <t>螺蛳粉</t>
+  </si>
+  <si>
+    <t>liuzhou@example.com</t>
+  </si>
+  <si>
+    <t>老干妈</t>
+  </si>
+  <si>
+    <t>风味豆豉辣椒酱</t>
+  </si>
+  <si>
+    <t>laoganma@example.com</t>
+  </si>
+  <si>
+    <t>南阳艾草制品供应链</t>
+  </si>
+  <si>
+    <t>中式养生</t>
+  </si>
+  <si>
+    <t>刮痧板</t>
+  </si>
+  <si>
+    <t>nanyang@example.com</t>
   </si>
 </sst>
 </file>
@@ -1208,15 +1685,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:G22"/>
+  <dimension ref="B1:H79"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
-    <col min="2" max="2" width="20.1826923076923" customWidth="1"/>
-    <col min="5" max="5" width="12.9230769230769"/>
-    <col min="6" max="6" width="31.7307692307692" customWidth="1"/>
+    <col min="2" max="2" width="23.5576923076923" customWidth="1"/>
+    <col min="3" max="3" width="14.0" customWidth="1"/>
+    <col min="4" max="4" width="17.1442307692308" customWidth="1"/>
+    <col min="5" max="5" width="20.5096153846154" customWidth="1"/>
+    <col min="6" max="6" width="25.7980769230769" customWidth="1"/>
+    <col min="7" max="7" width="30.0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7">
+    <row r="1" spans="2:8">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1235,374 +1715,1884 @@
       <c r="G1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="2:7">
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8">
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1">
+        <v>2.50</v>
+      </c>
+      <c r="F2">
+        <v>13800138000</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="E2">
-        <v>13521574937</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="2:7">
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1">
+        <v>3.20</v>
+      </c>
+      <c r="F3">
+        <v>13800138000</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1">
-        <v>1.1</v>
-      </c>
-      <c r="E3">
-        <v>13521574938</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="2:7">
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5.80</v>
+      </c>
+      <c r="F4">
+        <v>13800138000</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="1">
-        <v>2.1</v>
-      </c>
-      <c r="E4">
-        <v>13521574939</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="C5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="2:7">
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3.1</v>
-      </c>
-      <c r="E5">
-        <v>13521574940</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7">
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1.90</v>
+      </c>
+      <c r="F5">
+        <v>13800138000</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8">
       <c r="B6" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1">
-        <v>4.1</v>
-      </c>
-      <c r="E6">
-        <v>13521574941</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1">
+        <v>12.50</v>
+      </c>
+      <c r="F6">
+        <v>13800138001</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8">
       <c r="B7" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1">
-        <v>5.1</v>
-      </c>
-      <c r="E7">
-        <v>13521574942</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="1">
+        <v>8.80</v>
+      </c>
+      <c r="F7">
+        <v>13800138001</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8">
       <c r="B8" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="E8">
-        <v>13521574943</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1">
+        <v>15.60</v>
+      </c>
+      <c r="F8">
+        <v>13800138001</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
       <c r="B9" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1">
-        <v>7.1</v>
-      </c>
-      <c r="E9">
-        <v>13521574944</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1">
+        <v>22.00</v>
+      </c>
+      <c r="F9">
+        <v>13800138001</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
       <c r="B10" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="E10">
-        <v>13521574945</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1">
+        <v>6.50</v>
+      </c>
+      <c r="F10">
+        <v>13800138002</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8">
       <c r="B11" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="E11">
-        <v>13521574946</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="1">
+        <v>9.90</v>
+      </c>
+      <c r="F11">
+        <v>13800138002</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
       <c r="B12" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="1">
-        <v>10.1</v>
-      </c>
-      <c r="E12">
-        <v>13521574947</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7">
+        <v>23</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="1">
+        <v>7.20</v>
+      </c>
+      <c r="F12">
+        <v>13800138002</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
       <c r="B13" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="1">
-        <v>11.1</v>
-      </c>
-      <c r="E13">
-        <v>13521574948</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="1">
+        <v>3.40</v>
+      </c>
+      <c r="F13">
+        <v>13800138002</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8">
       <c r="B14" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="1">
-        <v>12.1</v>
-      </c>
-      <c r="E14">
-        <v>13521574949</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="1">
+        <v>128.00</v>
+      </c>
+      <c r="F14">
+        <v>13800138003</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
       <c r="B15" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="1">
-        <v>13.1</v>
-      </c>
-      <c r="E15">
-        <v>13521574950</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="1">
+        <v>96.00</v>
+      </c>
+      <c r="F15">
+        <v>13800138003</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
       <c r="B16" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="1">
-        <v>14.1</v>
-      </c>
-      <c r="E16">
-        <v>13521574951</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="1">
+        <v>158.00</v>
+      </c>
+      <c r="F16">
+        <v>13800138003</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8">
       <c r="B17" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="1">
-        <v>15.1</v>
-      </c>
-      <c r="E17">
-        <v>13521574952</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="1">
+        <v>42.00</v>
+      </c>
+      <c r="F17">
+        <v>13800138003</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8">
       <c r="B18" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="1">
-        <v>16.1</v>
-      </c>
-      <c r="E18">
-        <v>13521574953</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6">
+        <v>37</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="1">
+        <v>88.00</v>
+      </c>
+      <c r="F18">
+        <v>13800138004</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8">
       <c r="B19" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="1">
-        <v>17.1</v>
-      </c>
-      <c r="E19">
-        <v>13521574954</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="1">
+        <v>120.00</v>
+      </c>
+      <c r="F19">
+        <v>13800138004</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8">
       <c r="B20" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="1">
-        <v>18.1</v>
-      </c>
-      <c r="E20">
-        <v>13521574955</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="1">
+        <v>260.00</v>
+      </c>
+      <c r="F20">
+        <v>13800138004</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8">
       <c r="B21" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="1">
-        <v>19.1</v>
-      </c>
-      <c r="E21">
-        <v>13521574956</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6">
-      <c r="D22" s="1">
-        <v>20.1</v>
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" s="1">
+        <v>56.00</v>
+      </c>
+      <c r="F21">
+        <v>13800138004</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8">
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="1">
+        <v>68.00</v>
+      </c>
+      <c r="F22">
+        <v>13800138005</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8">
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="1">
+        <v>32.50</v>
+      </c>
+      <c r="F23">
+        <v>13800138005</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8">
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="1">
+        <v>18.00</v>
+      </c>
+      <c r="F24">
+        <v>13800138005</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8">
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="1">
+        <v>45.00</v>
+      </c>
+      <c r="F25">
+        <v>13800138005</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H25" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8">
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="1">
+        <v>14.00</v>
+      </c>
+      <c r="F26">
+        <v>13800138006</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8">
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" t="s">
+        <v>55</v>
+      </c>
+      <c r="E27" s="1">
+        <v>36.00</v>
+      </c>
+      <c r="F27">
+        <v>13800138006</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H27" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8">
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" s="1">
+        <v>24.00</v>
+      </c>
+      <c r="F28">
+        <v>13800138006</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8">
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="1">
+        <v>48.00</v>
+      </c>
+      <c r="F29">
+        <v>13800138006</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H29" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8">
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30" s="1">
+        <v>58.00</v>
+      </c>
+      <c r="F30">
+        <v>13800138007</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8">
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" t="s">
+        <v>59</v>
+      </c>
+      <c r="D31" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="1">
+        <v>46.00</v>
+      </c>
+      <c r="F31">
+        <v>13800138007</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8">
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" s="1">
+        <v>168.00</v>
+      </c>
+      <c r="F32">
+        <v>13800138007</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8">
+      <c r="B33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" s="1">
+        <v>210.00</v>
+      </c>
+      <c r="F33">
+        <v>13800138007</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H33" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8">
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" t="s">
+        <v>67</v>
+      </c>
+      <c r="E34" s="1">
+        <v>12.00</v>
+      </c>
+      <c r="F34">
+        <v>13800138008</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8">
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E35" s="1">
+        <v>26.00</v>
+      </c>
+      <c r="F35">
+        <v>13800138008</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8">
+      <c r="B36" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" t="s">
+        <v>66</v>
+      </c>
+      <c r="D36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36" s="1">
+        <v>34.00</v>
+      </c>
+      <c r="F36">
+        <v>13800138008</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H36" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8">
+      <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" t="s">
+        <v>71</v>
+      </c>
+      <c r="E37" s="1">
+        <v>28.00</v>
+      </c>
+      <c r="F37">
+        <v>13800138008</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H37" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8">
+      <c r="B38" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="1">
+        <v>76.00</v>
+      </c>
+      <c r="F38">
+        <v>13800138009</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H38" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8">
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" t="s">
+        <v>73</v>
+      </c>
+      <c r="D39" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" s="1">
+        <v>32.00</v>
+      </c>
+      <c r="F39">
+        <v>13800138009</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8">
+      <c r="B40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E40" s="1">
+        <v>24.50</v>
+      </c>
+      <c r="F40">
+        <v>13800138009</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H40" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8">
+      <c r="B41" t="s">
+        <v>72</v>
+      </c>
+      <c r="C41" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" t="s">
+        <v>78</v>
+      </c>
+      <c r="E41" s="1">
+        <v>88.00</v>
+      </c>
+      <c r="F41">
+        <v>13800138009</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H41" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8">
+      <c r="B42" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" t="s">
+        <v>81</v>
+      </c>
+      <c r="E42" s="1">
+        <v>42.00</v>
+      </c>
+      <c r="F42">
+        <v>13800138010</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H42" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8">
+      <c r="B43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" t="s">
+        <v>83</v>
+      </c>
+      <c r="E43" s="1">
+        <v>38.00</v>
+      </c>
+      <c r="F43">
+        <v>13800138010</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H43" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8">
+      <c r="B44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" t="s">
+        <v>84</v>
+      </c>
+      <c r="E44" s="1">
+        <v>96.00</v>
+      </c>
+      <c r="F44">
+        <v>13800138010</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H44" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8">
+      <c r="B45" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" t="s">
+        <v>85</v>
+      </c>
+      <c r="E45" s="1">
+        <v>118.00</v>
+      </c>
+      <c r="F45">
+        <v>13800138010</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H45" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8">
+      <c r="B46" t="s">
+        <v>86</v>
+      </c>
+      <c r="C46" t="s">
+        <v>87</v>
+      </c>
+      <c r="D46" t="s">
+        <v>88</v>
+      </c>
+      <c r="E46" s="1">
+        <v>36.00</v>
+      </c>
+      <c r="F46">
+        <v>13800138011</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H46" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8">
+      <c r="B47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" t="s">
+        <v>87</v>
+      </c>
+      <c r="D47" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" s="1">
+        <v>52.00</v>
+      </c>
+      <c r="F47">
+        <v>13800138011</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H47" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="2:8">
+      <c r="B48" t="s">
+        <v>86</v>
+      </c>
+      <c r="C48" t="s">
+        <v>87</v>
+      </c>
+      <c r="D48" t="s">
+        <v>91</v>
+      </c>
+      <c r="E48" s="1">
+        <v>45.00</v>
+      </c>
+      <c r="F48">
+        <v>13800138011</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H48" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8">
+      <c r="B49" t="s">
+        <v>86</v>
+      </c>
+      <c r="C49" t="s">
+        <v>87</v>
+      </c>
+      <c r="D49" t="s">
+        <v>92</v>
+      </c>
+      <c r="E49" s="1">
+        <v>18.50</v>
+      </c>
+      <c r="F49">
+        <v>13800138011</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H49" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8">
+      <c r="B50" t="s">
+        <v>93</v>
+      </c>
+      <c r="C50" t="s">
+        <v>94</v>
+      </c>
+      <c r="D50" t="s">
+        <v>95</v>
+      </c>
+      <c r="E50" s="1">
+        <v>28.00</v>
+      </c>
+      <c r="F50">
+        <v>13800138012</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8">
+      <c r="B51" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" t="s">
+        <v>94</v>
+      </c>
+      <c r="D51" t="s">
+        <v>97</v>
+      </c>
+      <c r="E51" s="1">
+        <v>16.50</v>
+      </c>
+      <c r="F51">
+        <v>13800138012</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H51" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8">
+      <c r="B52" t="s">
+        <v>93</v>
+      </c>
+      <c r="C52" t="s">
+        <v>94</v>
+      </c>
+      <c r="D52" t="s">
+        <v>98</v>
+      </c>
+      <c r="E52" s="1">
+        <v>12.80</v>
+      </c>
+      <c r="F52">
+        <v>13800138012</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8">
+      <c r="B53" t="s">
+        <v>93</v>
+      </c>
+      <c r="C53" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" t="s">
+        <v>99</v>
+      </c>
+      <c r="E53" s="1">
+        <v>9.60</v>
+      </c>
+      <c r="F53">
+        <v>13800138012</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8">
+      <c r="B54" t="s">
+        <v>100</v>
+      </c>
+      <c r="C54" t="s">
+        <v>101</v>
+      </c>
+      <c r="D54" t="s">
+        <v>102</v>
+      </c>
+      <c r="E54" s="1">
+        <v>6.80</v>
+      </c>
+      <c r="F54">
+        <v>13800138013</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8">
+      <c r="B55" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" t="s">
+        <v>101</v>
+      </c>
+      <c r="D55" t="s">
+        <v>104</v>
+      </c>
+      <c r="E55" s="1">
+        <v>8.50</v>
+      </c>
+      <c r="F55">
+        <v>13800138013</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8">
+      <c r="B56" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" t="s">
+        <v>101</v>
+      </c>
+      <c r="D56" t="s">
+        <v>105</v>
+      </c>
+      <c r="E56" s="1">
+        <v>4.20</v>
+      </c>
+      <c r="F56">
+        <v>13800138013</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8">
+      <c r="B57" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" t="s">
+        <v>101</v>
+      </c>
+      <c r="D57" t="s">
+        <v>106</v>
+      </c>
+      <c r="E57" s="1">
+        <v>3.60</v>
+      </c>
+      <c r="F57">
+        <v>13800138013</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58" spans="2:8">
+      <c r="B58" t="s">
+        <v>107</v>
+      </c>
+      <c r="C58" t="s">
+        <v>108</v>
+      </c>
+      <c r="D58" t="s">
+        <v>109</v>
+      </c>
+      <c r="E58" s="1">
+        <v>52.00</v>
+      </c>
+      <c r="F58">
+        <v>13800138014</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H58" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8">
+      <c r="B59" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" t="s">
+        <v>108</v>
+      </c>
+      <c r="D59" t="s">
+        <v>111</v>
+      </c>
+      <c r="E59" s="1">
+        <v>68.00</v>
+      </c>
+      <c r="F59">
+        <v>13800138014</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H59" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="2:8">
+      <c r="B60" t="s">
+        <v>107</v>
+      </c>
+      <c r="C60" t="s">
+        <v>108</v>
+      </c>
+      <c r="D60" t="s">
+        <v>112</v>
+      </c>
+      <c r="E60" s="1">
+        <v>46.00</v>
+      </c>
+      <c r="F60">
+        <v>13800138014</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H60" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8">
+      <c r="B61" t="s">
+        <v>107</v>
+      </c>
+      <c r="C61" t="s">
+        <v>108</v>
+      </c>
+      <c r="D61" t="s">
+        <v>113</v>
+      </c>
+      <c r="E61" s="1">
+        <v>22.00</v>
+      </c>
+      <c r="F61">
+        <v>13800138014</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H61" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62" spans="2:8">
+      <c r="B62" t="s">
+        <v>114</v>
+      </c>
+      <c r="C62" t="s">
+        <v>115</v>
+      </c>
+      <c r="D62" t="s">
+        <v>116</v>
+      </c>
+      <c r="E62" s="1">
+        <v>79.00</v>
+      </c>
+      <c r="F62">
+        <v>13800138015</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" spans="2:8">
+      <c r="B63" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" t="s">
+        <v>115</v>
+      </c>
+      <c r="D63" t="s">
+        <v>119</v>
+      </c>
+      <c r="E63" s="1">
+        <v>3999.00</v>
+      </c>
+      <c r="F63">
+        <v>13800138016</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8">
+      <c r="B64" t="s">
+        <v>69</v>
+      </c>
+      <c r="C64" t="s">
+        <v>115</v>
+      </c>
+      <c r="D64" t="s">
+        <v>121</v>
+      </c>
+      <c r="E64" s="1">
+        <v>1699.00</v>
+      </c>
+      <c r="F64">
+        <v>13800138017</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="2:8">
+      <c r="B65" t="s">
+        <v>123</v>
+      </c>
+      <c r="C65" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" t="s">
+        <v>125</v>
+      </c>
+      <c r="E65" s="1">
+        <v>2599.00</v>
+      </c>
+      <c r="F65">
+        <v>13800138018</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8">
+      <c r="B66" t="s">
+        <v>127</v>
+      </c>
+      <c r="C66" t="s">
+        <v>124</v>
+      </c>
+      <c r="D66" t="s">
+        <v>128</v>
+      </c>
+      <c r="E66" s="1">
+        <v>2199.00</v>
+      </c>
+      <c r="F66">
+        <v>13800138019</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H66" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="67" spans="2:8">
+      <c r="B67" t="s">
+        <v>130</v>
+      </c>
+      <c r="C67" t="s">
+        <v>124</v>
+      </c>
+      <c r="D67" t="s">
+        <v>131</v>
+      </c>
+      <c r="E67" s="1">
+        <v>3280.00</v>
+      </c>
+      <c r="F67">
+        <v>13800138020</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="H67" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8">
+      <c r="B68" t="s">
+        <v>133</v>
+      </c>
+      <c r="C68" t="s">
+        <v>134</v>
+      </c>
+      <c r="D68" t="s">
+        <v>135</v>
+      </c>
+      <c r="E68" s="1">
+        <v>189.00</v>
+      </c>
+      <c r="F68">
+        <v>13800138021</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H68" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8">
+      <c r="B69" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" t="s">
+        <v>134</v>
+      </c>
+      <c r="D69" t="s">
+        <v>138</v>
+      </c>
+      <c r="E69" s="1">
+        <v>19.90</v>
+      </c>
+      <c r="F69">
+        <v>13800138022</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H69" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8">
+      <c r="B70" t="s">
+        <v>137</v>
+      </c>
+      <c r="C70" t="s">
+        <v>134</v>
+      </c>
+      <c r="D70" t="s">
+        <v>140</v>
+      </c>
+      <c r="E70" s="1">
+        <v>29.90</v>
+      </c>
+      <c r="F70">
+        <v>13800138022</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H70" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8">
+      <c r="B71" t="s">
+        <v>141</v>
+      </c>
+      <c r="C71" t="s">
+        <v>142</v>
+      </c>
+      <c r="D71" t="s">
+        <v>143</v>
+      </c>
+      <c r="E71" s="1">
+        <v>69.00</v>
+      </c>
+      <c r="F71">
+        <v>13800138023</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H71" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8">
+      <c r="B72" t="s">
+        <v>145</v>
+      </c>
+      <c r="C72" t="s">
+        <v>142</v>
+      </c>
+      <c r="D72" t="s">
+        <v>146</v>
+      </c>
+      <c r="E72" s="1">
+        <v>899.00</v>
+      </c>
+      <c r="F72">
+        <v>13800138024</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="H72" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="73" spans="2:8">
+      <c r="B73" t="s">
+        <v>148</v>
+      </c>
+      <c r="C73" t="s">
+        <v>149</v>
+      </c>
+      <c r="D73" t="s">
+        <v>150</v>
+      </c>
+      <c r="E73" s="1">
+        <v>45.00</v>
+      </c>
+      <c r="F73">
+        <v>13800138025</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H73" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="74" spans="2:8">
+      <c r="B74" t="s">
+        <v>148</v>
+      </c>
+      <c r="C74" t="s">
+        <v>149</v>
+      </c>
+      <c r="D74" t="s">
+        <v>152</v>
+      </c>
+      <c r="E74" s="1">
+        <v>32.50</v>
+      </c>
+      <c r="F74">
+        <v>13800138025</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H74" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="75" spans="2:8">
+      <c r="B75" t="s">
+        <v>148</v>
+      </c>
+      <c r="C75" t="s">
+        <v>149</v>
+      </c>
+      <c r="D75" t="s">
+        <v>153</v>
+      </c>
+      <c r="E75" s="1">
+        <v>680.00</v>
+      </c>
+      <c r="F75">
+        <v>13800138025</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H75" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="76" spans="2:8">
+      <c r="B76" t="s">
+        <v>154</v>
+      </c>
+      <c r="C76" t="s">
+        <v>155</v>
+      </c>
+      <c r="D76" t="s">
+        <v>156</v>
+      </c>
+      <c r="E76" s="1">
+        <v>299.00</v>
+      </c>
+      <c r="F76">
+        <v>13800138026</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H76" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="77" spans="2:8">
+      <c r="B77" t="s">
+        <v>158</v>
+      </c>
+      <c r="C77" t="s">
+        <v>159</v>
+      </c>
+      <c r="D77" t="s">
+        <v>160</v>
+      </c>
+      <c r="E77" s="1">
+        <v>12.90</v>
+      </c>
+      <c r="F77">
+        <v>13800138027</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H77" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="78" spans="2:8">
+      <c r="B78" t="s">
+        <v>162</v>
+      </c>
+      <c r="C78" t="s">
+        <v>159</v>
+      </c>
+      <c r="D78" t="s">
+        <v>163</v>
+      </c>
+      <c r="E78" s="1">
+        <v>9.90</v>
+      </c>
+      <c r="F78">
+        <v>13800138028</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="H78" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="79" spans="2:8">
+      <c r="B79" t="s">
+        <v>165</v>
+      </c>
+      <c r="C79" t="s">
+        <v>166</v>
+      </c>
+      <c r="D79" t="s">
+        <v>167</v>
+      </c>
+      <c r="E79" s="1">
+        <v>39.00</v>
+      </c>
+      <c r="F79">
+        <v>13800138029</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="H79" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F3" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F4" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F5" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F6" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F7" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F8" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F9" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F10" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F11" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F12" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F13" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F14" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F15" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F16" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F17" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F18" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F19" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F20" r:id="rId1" display="wahah@qq.com"/>
-    <hyperlink ref="F21" r:id="rId1" display="wahah@qq.com"/>
+    <hyperlink ref="G2" r:id="rId9" display="huadong@example.com"/>
+    <hyperlink ref="G3" r:id="rId9" display="huadong@example.com"/>
+    <hyperlink ref="G4" r:id="rId9" display="huadong@example.com"/>
+    <hyperlink ref="G5" r:id="rId9" display="huadong@example.com"/>
+    <hyperlink ref="G6" r:id="rId2" display="chuanyu@example.com"/>
+    <hyperlink ref="G7" r:id="rId2" display="chuanyu@example.com"/>
+    <hyperlink ref="G8" r:id="rId2" display="chuanyu@example.com"/>
+    <hyperlink ref="G9" r:id="rId2" display="chuanyu@example.com"/>
+    <hyperlink ref="G10" r:id="rId12" display="lingnan@example.com"/>
+    <hyperlink ref="G11" r:id="rId12" display="lingnan@example.com"/>
+    <hyperlink ref="G12" r:id="rId12" display="lingnan@example.com"/>
+    <hyperlink ref="G13" r:id="rId12" display="lingnan@example.com"/>
+    <hyperlink ref="G14" r:id="rId19" display="qilu@example.com"/>
+    <hyperlink ref="G15" r:id="rId19" display="qilu@example.com"/>
+    <hyperlink ref="G16" r:id="rId19" display="qilu@example.com"/>
+    <hyperlink ref="G17" r:id="rId19" display="qilu@example.com"/>
+    <hyperlink ref="G18" r:id="rId28" display="yungui@example.com"/>
+    <hyperlink ref="G19" r:id="rId28" display="yungui@example.com"/>
+    <hyperlink ref="G20" r:id="rId28" display="yungui@example.com"/>
+    <hyperlink ref="G21" r:id="rId28" display="yungui@example.com"/>
+    <hyperlink ref="G22" r:id="rId15" display="minnan@example.com"/>
+    <hyperlink ref="G23" r:id="rId15" display="minnan@example.com"/>
+    <hyperlink ref="G24" r:id="rId15" display="minnan@example.com"/>
+    <hyperlink ref="G25" r:id="rId15" display="minnan@example.com"/>
+    <hyperlink ref="G26" r:id="rId23" display="xiange@example.com"/>
+    <hyperlink ref="G27" r:id="rId23" display="xiange@example.com"/>
+    <hyperlink ref="G28" r:id="rId23" display="xiange@example.com"/>
+    <hyperlink ref="G29" r:id="rId23" display="xiange@example.com"/>
+    <hyperlink ref="G30" r:id="rId8" display="huabei@example.com"/>
+    <hyperlink ref="G31" r:id="rId8" display="huabei@example.com"/>
+    <hyperlink ref="G32" r:id="rId8" display="huabei@example.com"/>
+    <hyperlink ref="G33" r:id="rId8" display="huabei@example.com"/>
+    <hyperlink ref="G34" r:id="rId4" display="dongbei@example.com"/>
+    <hyperlink ref="G35" r:id="rId4" display="dongbei@example.com"/>
+    <hyperlink ref="G36" r:id="rId4" display="dongbei@example.com"/>
+    <hyperlink ref="G37" r:id="rId4" display="dongbei@example.com"/>
+    <hyperlink ref="G38" r:id="rId10" display="jiangzhe@example.com"/>
+    <hyperlink ref="G39" r:id="rId10" display="jiangzhe@example.com"/>
+    <hyperlink ref="G40" r:id="rId10" display="jiangzhe@example.com"/>
+    <hyperlink ref="G41" r:id="rId10" display="jiangzhe@example.com"/>
+    <hyperlink ref="G42" r:id="rId25" display="xibei@example.com"/>
+    <hyperlink ref="G43" r:id="rId25" display="xibei@example.com"/>
+    <hyperlink ref="G44" r:id="rId25" display="xibei@example.com"/>
+    <hyperlink ref="G45" r:id="rId25" display="xibei@example.com"/>
+    <hyperlink ref="G46" r:id="rId30" display="zhusanjiao@example.com"/>
+    <hyperlink ref="G47" r:id="rId30" display="zhusanjiao@example.com"/>
+    <hyperlink ref="G48" r:id="rId30" display="zhusanjiao@example.com"/>
+    <hyperlink ref="G49" r:id="rId30" display="zhusanjiao@example.com"/>
+    <hyperlink ref="G50" r:id="rId29" display="zhongyuan@example.com"/>
+    <hyperlink ref="G51" r:id="rId29" display="zhongyuan@example.com"/>
+    <hyperlink ref="G52" r:id="rId29" display="zhongyuan@example.com"/>
+    <hyperlink ref="G53" r:id="rId29" display="zhongyuan@example.com"/>
+    <hyperlink ref="G54" r:id="rId7" display="hainan@example.com"/>
+    <hyperlink ref="G55" r:id="rId7" display="hainan@example.com"/>
+    <hyperlink ref="G56" r:id="rId7" display="hainan@example.com"/>
+    <hyperlink ref="G57" r:id="rId7" display="hainan@example.com"/>
+    <hyperlink ref="G58" r:id="rId22" display="wannan@example.com"/>
+    <hyperlink ref="G59" r:id="rId22" display="wannan@example.com"/>
+    <hyperlink ref="G60" r:id="rId22" display="wannan@example.com"/>
+    <hyperlink ref="G61" r:id="rId22" display="wannan@example.com"/>
+    <hyperlink ref="G62" r:id="rId1" display="anker@example.com"/>
+    <hyperlink ref="G63" r:id="rId3" display="dji@example.com"/>
+    <hyperlink ref="G64" r:id="rId24" display="xiaomi@example.com"/>
+    <hyperlink ref="G65" r:id="rId5" display="ecoflow@example.com"/>
+    <hyperlink ref="G66" r:id="rId20" display="segway@example.com"/>
+    <hyperlink ref="G67" r:id="rId21" display="shenzhen-clean@example.com"/>
+    <hyperlink ref="G68" r:id="rId26" display="xuchang@example.com"/>
+    <hyperlink ref="G69" r:id="rId27" display="yiwu@example.com"/>
+    <hyperlink ref="G70" r:id="rId27" display="yiwu@example.com"/>
+    <hyperlink ref="G71" r:id="rId18" display="popmart@example.com"/>
+    <hyperlink ref="G72" r:id="rId6" display="goodbaby@example.com"/>
+    <hyperlink ref="G73" r:id="rId17" display="ningbo@example.com"/>
+    <hyperlink ref="G74" r:id="rId17" display="ningbo@example.com"/>
+    <hyperlink ref="G75" r:id="rId17" display="ningbo@example.com"/>
+    <hyperlink ref="G76" r:id="rId14" display="midea@example.com"/>
+    <hyperlink ref="G77" r:id="rId13" display="liuzhou@example.com"/>
+    <hyperlink ref="G78" r:id="rId11" display="laoganma@example.com"/>
+    <hyperlink ref="G79" r:id="rId16" display="nanyang@example.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>